<commit_message>
docs(agrupamento): modelo P38 solo/composto + export Excel actualizado
Documenta lógica portal vs Leroy Merlin. Regenera estudo hierarquia com
barra roscada e fixação na LINHA PARAFUSO.

Co-authored-by: joaoandreriberopacheco-netizen <joaoandreriberopacheco-netizen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/exports/P38-sku-hierarquia-estudo.xlsx
+++ b/docs/exports/P38-sku-hierarquia-estudo.xlsx
@@ -5851,16 +5851,16 @@
     <t>CERAM BOLD SEMI 50X50 TRAGEGO BG</t>
   </si>
   <si>
+    <t>BURITI BEGE PEI 3 (2,00M²/ CX)</t>
+  </si>
+  <si>
+    <t>PISO 45X45 BURITI BEGE PEI 3 (2,00M²/ CX)</t>
+  </si>
+  <si>
     <t>TRAFEGO BEGE PEI 5 (2,00M²/ CX)</t>
   </si>
   <si>
     <t>PISO 50X50 TRAFEGO BEGE PEI 5 (2,00M²/ CX)</t>
-  </si>
-  <si>
-    <t>BURITI BEGE PEI 3 (2,00M²/ CX)</t>
-  </si>
-  <si>
-    <t>PISO 45X45 BURITI BEGE PEI 3 (2,00M²/ CX)</t>
   </si>
   <si>
     <t>PQM-Q2L</t>
@@ -33965,7 +33965,7 @@
         <v>1162</v>
       </c>
       <c r="I501" t="s">
-        <v>1943</v>
+        <v>1226</v>
       </c>
       <c r="J501" t="s">
         <v>1946</v>
@@ -34006,7 +34006,7 @@
         <v>1162</v>
       </c>
       <c r="I502" t="s">
-        <v>1226</v>
+        <v>1943</v>
       </c>
       <c r="J502" t="s">
         <v>1948</v>

</xml_diff>